<commit_message>
v1.37.6: Enhance calendar festivo management with override and class sync
- Introduce `lectivo_override` status for `festivos_calendario`, allowing users
  to explicitly mark a day as teaching even if it's defined as a holiday in
  `config.json`.
- When a class is updated from non-teaching (`es_no_lectivo=1`) to teaching
  (`es_no_lectivo=0`), automatically remove the day from `festivos_calendario`
  and clean up any other placeholder non-teaching classes for that day.
- Update the calendar UI (popup, day rendering, festivos list) to correctly
  display and manage these `lectivo_override` days.
- Updates academic calendar `calendario_academico_26_27.xlsx`.
- Updates application version to 1.37.6.
</commit_message>
<xml_diff>
--- a/config/calendario_academico_26_27.xlsx
+++ b/config/calendario_academico_26_27.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jfrutos/Library/CloudStorage/Dropbox/PASAR A DISCO/COORDINACION GIM/Janux/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B89B5F-D5F3-0E4B-9BF3-FA364C3064BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70EBC44E-3EEB-E94E-8D82-D18F4B57822F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="17920" windowHeight="20320" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="45">
   <si>
     <t>Festivos y Días No Lectivos</t>
   </si>
@@ -376,7 +376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -463,13 +463,22 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -845,7 +854,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="31" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="29"/>
@@ -918,7 +927,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="32" t="s">
         <v>38</v>
       </c>
       <c r="B15" s="29"/>
@@ -936,7 +945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -972,7 +981,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="15">
-        <v>46283</v>
+        <v>46297</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>6</v>
@@ -1051,93 +1060,129 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="15">
-        <v>46458</v>
+    <row r="9" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="35">
+        <v>46379</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="15">
-        <v>46465</v>
+      <c r="D9" s="33"/>
+    </row>
+    <row r="10" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="35">
+        <v>46380</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="15">
-        <v>46475</v>
+        <v>6</v>
+      </c>
+      <c r="D10" s="33"/>
+    </row>
+    <row r="11" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="35">
+        <v>46381</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="10"/>
+      <c r="D11" s="33"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="15">
-        <v>46476</v>
+        <v>46458</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="10"/>
+      <c r="D12" s="10" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B13" s="15">
-        <v>46415</v>
+        <v>46465</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="27" t="s">
-        <v>44</v>
+        <v>8</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B14" s="15">
-        <v>46547</v>
+        <v>46475</v>
       </c>
       <c r="C14" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="27"/>
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="15">
+        <v>46476</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="15">
+        <v>46415</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="15">
+        <v>46547</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C3:C201" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="C3:C204" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"festivo,no_lectivo"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="A3:A300" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="A3:A303" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"1C,2C,ENERO,JUNIO,EXTRAORD"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1184,7 +1229,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="30" t="s">
         <v>43</v>
       </c>
       <c r="B5" s="29"/>

</xml_diff>